<commit_message>
Use hatched fills for yield-loss blocks to match whiteboard sketch
The gross-kill portion above each slaughterhouse's net block is now a
diagonal hatch in the same hue instead of a pale tint, matching the
planning sketch of the capacity-vs-demand graph.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014fnah7533XZizagq8i6MTs
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/Supplier_Capacity_Inputs.xlsx
+++ b/PVA second supplier initiative/Supplier_Capacity_Inputs.xlsx
@@ -119,7 +119,7 @@
     <t xml:space="preserve">Slaughterhouse Capacity vs Tissue Demand per Quarter</t>
   </si>
   <si>
-    <t xml:space="preserve">Net = harvested pigs (Sheet1!J16:J19 = gross kill x wtd spec yield x wtd harvest yield). Yield loss = gross - net, drawn as the pale extension of each block. Demand = tissue units consumed per quarter (Sheet1!L10:P13), assuming 1 tissue = 1 pig equivalent (per request). Capacity is flat across quarters because Sheet1 gives a single weekly kill rate (x13 wks/qtr). All cells link to Sheet1.</t>
+    <t xml:space="preserve">Net = harvested pigs (Sheet1!J16:J19 = gross kill x wtd spec yield x wtd harvest yield). Yield loss = gross - net, drawn as the hatched extension of each block. Demand = tissue units consumed per quarter (Sheet1!L10:P13), assuming 1 tissue = 1 pig equivalent (per request). Capacity is flat across quarters because Sheet1 gives a single weekly kill rate (x13 wks/qtr). All cells link to Sheet1.</t>
   </si>
   <si>
     <t xml:space="preserve">Series</t>
@@ -138,11 +138,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="0%"/>
-    <numFmt numFmtId="166" formatCode="0.00%"/>
-    <numFmt numFmtId="167" formatCode="#,##0"/>
+    <numFmt numFmtId="165" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="0%"/>
+    <numFmt numFmtId="167" formatCode="0.00%"/>
+    <numFmt numFmtId="168" formatCode="#,##0"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -288,10 +289,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -300,23 +297,27 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -340,11 +341,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -374,15 +375,15 @@
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBFBF"/>
-      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF8B8B8B"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FFE34948"/>
-      <rgbColor rgb="FFFAE2B3"/>
-      <rgbColor rgb="FFD9D9D9"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFE87BA4"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFBFD6F3"/>
+      <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -393,12 +394,12 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFBBE7D7"/>
+      <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFF9D2C2"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF2A78D6"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -406,7 +407,7 @@
       <rgbColor rgb="FFEDA100"/>
       <rgbColor rgb="FFEB6834"/>
       <rgbColor rgb="FF595959"/>
-      <rgbColor rgb="FFB3B3B3"/>
+      <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF1BAF7A"/>
       <rgbColor rgb="FF0B0B0B"/>
@@ -446,7 +447,7 @@
                 </a:solidFill>
                 <a:latin typeface="Aptos Narrow"/>
               </a:rPr>
-              <a:t>Net harvested capacity (solid) vs gross kill (pale) vs total tissue demand</a:t>
+              <a:t>Net harvested capacity (solid) vs gross kill (hatched) vs total tissue demand</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -579,9 +580,14 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="bfd6f3"/>
-            </a:solidFill>
+            <a:pattFill prst="wdUpDiag">
+              <a:fgClr>
+                <a:srgbClr val="2a78d6"/>
+              </a:fgClr>
+              <a:bgClr>
+                <a:srgbClr val="ffffff"/>
+              </a:bgClr>
+            </a:pattFill>
             <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="ffffff"/>
@@ -777,9 +783,14 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="f9d2c2"/>
-            </a:solidFill>
+            <a:pattFill prst="wdUpDiag">
+              <a:fgClr>
+                <a:srgbClr val="eb6834"/>
+              </a:fgClr>
+              <a:bgClr>
+                <a:srgbClr val="ffffff"/>
+              </a:bgClr>
+            </a:pattFill>
             <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="ffffff"/>
@@ -975,9 +986,14 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="bbe7d7"/>
-            </a:solidFill>
+            <a:pattFill prst="wdUpDiag">
+              <a:fgClr>
+                <a:srgbClr val="1baf7a"/>
+              </a:fgClr>
+              <a:bgClr>
+                <a:srgbClr val="ffffff"/>
+              </a:bgClr>
+            </a:pattFill>
             <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="ffffff"/>
@@ -1173,9 +1189,14 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="fae2b3"/>
-            </a:solidFill>
+            <a:pattFill prst="wdUpDiag">
+              <a:fgClr>
+                <a:srgbClr val="eda100"/>
+              </a:fgClr>
+              <a:bgClr>
+                <a:srgbClr val="ffffff"/>
+              </a:bgClr>
+            </a:pattFill>
             <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="ffffff"/>
@@ -1259,8 +1280,8 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="63113231"/>
-        <c:axId val="66431258"/>
+        <c:axId val="313599"/>
+        <c:axId val="20721379"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1381,11 +1402,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="63113231"/>
-        <c:axId val="66431258"/>
+        <c:axId val="313599"/>
+        <c:axId val="20721379"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="63113231"/>
+        <c:axId val="313599"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1430,10 +1451,11 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln w="0">
+          <a:ln w="12600">
             <a:solidFill>
-              <a:srgbClr val="b3b3b3"/>
+              <a:srgbClr val="8b8b8b"/>
             </a:solidFill>
+            <a:round/>
           </a:ln>
         </c:spPr>
         <c:txPr>
@@ -1450,7 +1472,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66431258"/>
+        <c:crossAx val="20721379"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1458,7 +1480,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="66431258"/>
+        <c:axId val="20721379"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1466,10 +1488,11 @@
         <c:axPos val="l"/>
         <c:majorGridlines>
           <c:spPr>
-            <a:ln w="0">
+            <a:ln w="12600">
               <a:solidFill>
-                <a:srgbClr val="b3b3b3"/>
+                <a:srgbClr val="8b8b8b"/>
               </a:solidFill>
+              <a:round/>
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
@@ -1512,10 +1535,11 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln w="0">
+          <a:ln w="12600">
             <a:solidFill>
-              <a:srgbClr val="b3b3b3"/>
+              <a:srgbClr val="8b8b8b"/>
             </a:solidFill>
+            <a:round/>
           </a:ln>
         </c:spPr>
         <c:txPr>
@@ -1532,7 +1556,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63113231"/>
+        <c:crossAx val="313599"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2027,8 +2051,8 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="1142564"/>
-        <c:axId val="95739965"/>
+        <c:axId val="96558933"/>
+        <c:axId val="73157146"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2581,11 +2605,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="1142564"/>
-        <c:axId val="95739965"/>
+        <c:axId val="96558933"/>
+        <c:axId val="73157146"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1142564"/>
+        <c:axId val="96558933"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2630,10 +2654,11 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln w="0">
+          <a:ln w="12600">
             <a:solidFill>
-              <a:srgbClr val="b3b3b3"/>
+              <a:srgbClr val="8b8b8b"/>
             </a:solidFill>
+            <a:round/>
           </a:ln>
         </c:spPr>
         <c:txPr>
@@ -2650,7 +2675,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95739965"/>
+        <c:crossAx val="73157146"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2658,7 +2683,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="95739965"/>
+        <c:axId val="73157146"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2666,10 +2691,11 @@
         <c:axPos val="l"/>
         <c:majorGridlines>
           <c:spPr>
-            <a:ln w="0">
+            <a:ln w="12600">
               <a:solidFill>
-                <a:srgbClr val="b3b3b3"/>
+                <a:srgbClr val="8b8b8b"/>
               </a:solidFill>
+              <a:round/>
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
@@ -2712,10 +2738,11 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln w="0">
+          <a:ln w="12600">
             <a:solidFill>
-              <a:srgbClr val="b3b3b3"/>
+              <a:srgbClr val="8b8b8b"/>
             </a:solidFill>
+            <a:round/>
           </a:ln>
         </c:spPr>
         <c:txPr>
@@ -2732,7 +2759,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1142564"/>
+        <c:crossAx val="96558933"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3029,231 +3056,231 @@
   <dimension ref="C3:S23"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="27.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="16.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="27.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="16.44"/>
   </cols>
   <sheetData>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C3" s="2" t="s">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L3" s="2" t="n">
+      <c r="L3" s="1" t="n">
         <v>666501</v>
       </c>
-      <c r="M3" s="1" t="n">
+      <c r="M3" s="0" t="n">
         <v>666502</v>
       </c>
-      <c r="N3" s="1" t="n">
+      <c r="N3" s="0" t="n">
         <v>666506</v>
       </c>
-      <c r="O3" s="1" t="n">
+      <c r="O3" s="0" t="n">
         <v>666541</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C4" s="2" t="n">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C4" s="1" t="n">
         <v>666035</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="1" t="n">
         <v>90</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="1" t="n">
         <v>90</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="1" t="n">
         <v>95</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="1" t="n">
         <v>90</v>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="I4" s="1" t="n">
         <v>80</v>
       </c>
-      <c r="L4" s="3" t="n">
+      <c r="L4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M4" s="3" t="n">
+      <c r="M4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N4" s="3" t="n">
+      <c r="N4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O4" s="3" t="n">
+      <c r="O4" s="2" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C5" s="2" t="s">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="1" t="n">
         <v>300</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="1" t="n">
         <v>320</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="1" t="n">
         <v>340</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>365</v>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="I5" s="1" t="n">
         <v>380</v>
       </c>
-      <c r="L5" s="3" t="n">
+      <c r="L5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M5" s="3" t="n">
+      <c r="M5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="3" t="n">
+      <c r="N5" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O5" s="3" t="n">
+      <c r="O5" s="2" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C6" s="2" t="n">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C6" s="1" t="n">
         <v>666052</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="1" t="n">
         <v>135</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="1" t="n">
         <v>120</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="1" t="n">
         <v>125</v>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>125</v>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="I6" s="1" t="n">
         <v>128</v>
       </c>
-      <c r="L6" s="3" t="n">
+      <c r="L6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M6" s="3" t="n">
+      <c r="M6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N6" s="3" t="n">
+      <c r="N6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="O6" s="3" t="n">
+      <c r="O6" s="2" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C7" s="2" t="n">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C7" s="1" t="n">
         <v>666069</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="1" t="n">
         <v>1800</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="1" t="n">
         <v>1950</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="1" t="n">
         <v>2050</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="1" t="n">
         <v>2075</v>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I7" s="1" t="n">
         <v>2050</v>
       </c>
-      <c r="L7" s="3" t="n">
+      <c r="L7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="M7" s="3" t="n">
+      <c r="M7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N7" s="3" t="n">
+      <c r="N7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O7" s="3" t="n">
+      <c r="O7" s="2" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="L9" s="2" t="s">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L9" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="M9" s="2" t="s">
+      <c r="M9" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="N9" s="2" t="s">
+      <c r="N9" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="O9" s="2" t="s">
+      <c r="O9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="P9" s="2" t="s">
+      <c r="P9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="R9" s="2" t="s">
+      <c r="R9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="S9" s="2" t="s">
+      <c r="S9" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K10" s="2" t="n">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K10" s="1" t="n">
         <v>666501</v>
       </c>
-      <c r="L10" s="1" t="n">
+      <c r="L10" s="3" t="n">
         <f aca="false" t="array" ref="L10:L10">SUM(E$4:E$7*$L$4:$L$7)</f>
         <v>2970</v>
       </c>
-      <c r="M10" s="1" t="n">
+      <c r="M10" s="3" t="n">
         <f aca="false" t="array" ref="M10:M10">SUM(F$4:F$7*$L$4:$L$7)</f>
         <v>3150</v>
       </c>
-      <c r="N10" s="1" t="n">
+      <c r="N10" s="3" t="n">
         <f aca="false" t="array" ref="N10:N10">SUM(G$4:G$7*$L$4:$L$7)</f>
         <v>3320</v>
       </c>
-      <c r="O10" s="1" t="n">
+      <c r="O10" s="3" t="n">
         <f aca="false" t="array" ref="O10:O10">SUM(H$4:H$7*$L$4:$L$7)</f>
         <v>3420</v>
       </c>
-      <c r="P10" s="1" t="n">
+      <c r="P10" s="3" t="n">
         <f aca="false" t="array" ref="P10:P10">SUM(I$4:I$7*$L$4:$L$7)</f>
         <v>3446</v>
       </c>
@@ -3264,27 +3291,27 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K11" s="2" t="n">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K11" s="1" t="n">
         <v>666502</v>
       </c>
-      <c r="L11" s="1" t="n">
+      <c r="L11" s="3" t="n">
         <f aca="false" t="array" ref="L11:L11">SUM(E$4:E$7*$M$4:$M$7)</f>
         <v>1800</v>
       </c>
-      <c r="M11" s="1" t="n">
+      <c r="M11" s="3" t="n">
         <f aca="false" t="array" ref="M11:M11">SUM(F$4:F$7*$M$4:$M$7)</f>
         <v>1950</v>
       </c>
-      <c r="N11" s="1" t="n">
+      <c r="N11" s="3" t="n">
         <f aca="false" t="array" ref="N11:N11">SUM(G$4:G$7*$M$4:$M$7)</f>
         <v>2050</v>
       </c>
-      <c r="O11" s="1" t="n">
+      <c r="O11" s="3" t="n">
         <f aca="false" t="array" ref="O11:O11">SUM(H$4:H$7*$M$4:$M$7)</f>
         <v>2075</v>
       </c>
-      <c r="P11" s="1" t="n">
+      <c r="P11" s="3" t="n">
         <f aca="false" t="array" ref="P11:P11">SUM(I$4:I$7*$M$4:$M$7)</f>
         <v>2050</v>
       </c>
@@ -3295,27 +3322,27 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K12" s="2" t="n">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K12" s="1" t="n">
         <v>666506</v>
       </c>
-      <c r="L12" s="1" t="n">
+      <c r="L12" s="3" t="n">
         <f aca="false" t="array" ref="L12:L12">SUM(E$4:E$7*$N$4:$N$7)</f>
         <v>735</v>
       </c>
-      <c r="M12" s="1" t="n">
+      <c r="M12" s="3" t="n">
         <f aca="false" t="array" ref="M12:M12">SUM(F$4:F$7*$N$4:$N$7)</f>
         <v>760</v>
       </c>
-      <c r="N12" s="1" t="n">
+      <c r="N12" s="3" t="n">
         <f aca="false" t="array" ref="N12:N12">SUM(G$4:G$7*$N$4:$N$7)</f>
         <v>805</v>
       </c>
-      <c r="O12" s="1" t="n">
+      <c r="O12" s="3" t="n">
         <f aca="false" t="array" ref="O12:O12">SUM(H$4:H$7*$N$4:$N$7)</f>
         <v>855</v>
       </c>
-      <c r="P12" s="1" t="n">
+      <c r="P12" s="3" t="n">
         <f aca="false" t="array" ref="P12:P12">SUM(I$4:I$7*$N$4:$N$7)</f>
         <v>888</v>
       </c>
@@ -3326,27 +3353,27 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K13" s="2" t="n">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K13" s="1" t="n">
         <v>666541</v>
       </c>
-      <c r="L13" s="1" t="n">
+      <c r="L13" s="3" t="n">
         <f aca="false" t="array" ref="L13:L13">SUM(E$4:E$7*$O$4:$O$7)</f>
         <v>1800</v>
       </c>
-      <c r="M13" s="1" t="n">
+      <c r="M13" s="3" t="n">
         <f aca="false" t="array" ref="M13:M13">SUM(F$4:F$7*$O$4:$O$7)</f>
         <v>1950</v>
       </c>
-      <c r="N13" s="1" t="n">
+      <c r="N13" s="3" t="n">
         <f aca="false" t="array" ref="N13:N13">SUM(G$4:G$7*$O$4:$O$7)</f>
         <v>2050</v>
       </c>
-      <c r="O13" s="1" t="n">
+      <c r="O13" s="3" t="n">
         <f aca="false" t="array" ref="O13:O13">SUM(H$4:H$7*$O$4:$O$7)</f>
         <v>2075</v>
       </c>
-      <c r="P13" s="1" t="n">
+      <c r="P13" s="3" t="n">
         <f aca="false" t="array" ref="P13:P13">SUM(I$4:I$7*$O$4:$O$7)</f>
         <v>2050</v>
       </c>
@@ -3357,8 +3384,8 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F14" s="1" t="n">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F14" s="0" t="n">
         <v>13</v>
       </c>
       <c r="H14" s="5" t="s">
@@ -3368,34 +3395,34 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E15" s="1" t="s">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E15" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="F15" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="G15" s="0" t="s">
         <v>18</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="I15" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J15" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D16" s="1" t="s">
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D16" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="E16" s="1" t="n">
+      <c r="E16" s="0" t="n">
         <v>2500</v>
       </c>
-      <c r="F16" s="1" t="n">
+      <c r="F16" s="0" t="n">
         <f aca="false">E16*$F$14</f>
         <v>32500</v>
       </c>
@@ -3416,14 +3443,14 @@
         <v>17220.7857529863</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D17" s="1" t="s">
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D17" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="E17" s="0" t="n">
         <v>180</v>
       </c>
-      <c r="F17" s="1" t="n">
+      <c r="F17" s="0" t="n">
         <f aca="false">E17*$F$14</f>
         <v>2340</v>
       </c>
@@ -3444,14 +3471,14 @@
         <v>1239.89657421501</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D18" s="1" t="s">
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D18" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="0" t="n">
         <v>150</v>
       </c>
-      <c r="F18" s="1" t="n">
+      <c r="F18" s="0" t="n">
         <f aca="false">E18*$F$14</f>
         <v>1950</v>
       </c>
@@ -3472,14 +3499,14 @@
         <v>1033.24714517918</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D19" s="1" t="s">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D19" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="E19" s="1" t="n">
+      <c r="E19" s="0" t="n">
         <v>400</v>
       </c>
-      <c r="F19" s="1" t="n">
+      <c r="F19" s="0" t="n">
         <f aca="false">E19*$F$14</f>
         <v>5200</v>
       </c>
@@ -3500,28 +3527,28 @@
         <v>2396.61114142236</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="I22" s="1" t="s">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I22" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="L22" s="1" t="s">
+      <c r="L22" s="0" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="I23" s="1" t="s">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I23" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="J23" s="1" t="s">
+      <c r="J23" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="K23" s="1" t="s">
+      <c r="K23" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="L23" s="1" t="s">
+      <c r="L23" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="M23" s="1" t="s">
+      <c r="M23" s="0" t="s">
         <v>30</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add stack-total labels above bars on Viz 1 and Viz 2 charts
Invisible label-carrier series print the four-house totals above each
stack (31,733 net at spec; 21,891 net harvested) and 41,990 above the
gross-kill shadow bars, with their legend entries suppressed. In-chart
label formats aligned to full integers to match how Excel renders them.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014fnah7533XZizagq8i6MTs
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/Supplier_Capacity_Inputs.xlsx
+++ b/PVA second supplier initiative/Supplier_Capacity_Inputs.xlsx
@@ -373,6 +373,13 @@
       <family val="2"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FF0B0B0B"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="9"/>
       <color rgb="FF595959"/>
       <name val="Aptos Narrow"/>
@@ -382,13 +389,6 @@
       <b val="true"/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="9"/>
-      <color rgb="FF0B0B0B"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
@@ -932,9 +932,9 @@
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008300"/>
       <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF459428"/>
+      <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF7F7F7F"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBFBF"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF889AAA"/>
@@ -963,7 +963,7 @@
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF2A78D6"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF4EA72E"/>
+      <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFEDA100"/>
       <rgbColor rgb="FFEB6834"/>
@@ -1114,7 +1114,7 @@
           <dLbls>
             <dLbl>
               <idx val="0"/>
-              <numFmt formatCode="#,##0.0,&quot;K&quot;"/>
+              <numFmt formatCode="#,##0"/>
               <dLblPos val="ctr"/>
               <showLegendKey val="0"/>
               <showVal val="1"/>
@@ -1123,7 +1123,7 @@
               <showPercent val="0"/>
               <showBubbleSize val="0"/>
             </dLbl>
-            <numFmt formatCode="#,##0.0,&quot;K&quot;"/>
+            <numFmt formatCode="#,##0"/>
             <txPr>
               <a:bodyPr/>
               <a:p>
@@ -1231,7 +1231,7 @@
           <dLbls>
             <dLbl>
               <idx val="0"/>
-              <numFmt formatCode="#,##0.0,&quot;K&quot;"/>
+              <numFmt formatCode="#,##0"/>
               <dLblPos val="ctr"/>
               <showLegendKey val="0"/>
               <showVal val="1"/>
@@ -1240,7 +1240,7 @@
               <showPercent val="0"/>
               <showBubbleSize val="0"/>
             </dLbl>
-            <numFmt formatCode="#,##0.0,&quot;K&quot;"/>
+            <numFmt formatCode="#,##0"/>
             <txPr>
               <a:bodyPr/>
               <a:p>
@@ -1331,7 +1331,7 @@
           <dLbls>
             <dLbl>
               <idx val="4"/>
-              <numFmt formatCode="#,##0.0,&quot;K&quot;"/>
+              <numFmt formatCode="#,##0"/>
               <dLblPos val="t"/>
               <showLegendKey val="0"/>
               <showVal val="1"/>
@@ -1340,7 +1340,7 @@
               <showPercent val="0"/>
               <showBubbleSize val="0"/>
             </dLbl>
-            <numFmt formatCode="#,##0.0,&quot;K&quot;"/>
+            <numFmt formatCode="#,##0"/>
             <txPr>
               <a:bodyPr/>
               <a:p>
@@ -1377,8 +1377,131 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <v>Total (label)</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <txPr>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0">
+                    <a:solidFill>
+                      <a:srgbClr val="0B0B0B"/>
+                    </a:solidFill>
+                    <a:latin typeface="Aptos Narrow"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="900" b="1" i="0">
+                  <a:solidFill>
+                    <a:srgbClr val="0B0B0B"/>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="t"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+          </dLbls>
+          <val>
+            <numRef>
+              <f>'Chart Data'!$B$9:$F$9</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
         <axId val="10"/>
         <axId val="200"/>
+      </lineChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <tx>
+            <v>Total (label)</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <txPr>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0">
+                    <a:solidFill>
+                      <a:srgbClr val="0B0B0B"/>
+                    </a:solidFill>
+                    <a:latin typeface="Aptos Narrow"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="900" b="1" i="0">
+                  <a:solidFill>
+                    <a:srgbClr val="0B0B0B"/>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="t"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+          </dLbls>
+          <val>
+            <numRef>
+              <f>'Chart Data'!$B$15:$F$15</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
       </lineChart>
       <catAx>
         <axId val="10"/>
@@ -1497,6 +1620,14 @@
       <legendPos val="b"/>
       <legendEntry>
         <idx val="0"/>
+        <delete val="1"/>
+      </legendEntry>
+      <legendEntry>
+        <idx val="6"/>
+        <delete val="1"/>
+      </legendEntry>
+      <legendEntry>
+        <idx val="7"/>
         <delete val="1"/>
       </legendEntry>
       <layout>
@@ -1704,7 +1835,7 @@
           <dLbls>
             <dLbl>
               <idx val="0"/>
-              <numFmt formatCode="#,##0.0,&quot;K&quot;"/>
+              <numFmt formatCode="#,##0"/>
               <dLblPos val="ctr"/>
               <showLegendKey val="0"/>
               <showVal val="1"/>
@@ -1713,7 +1844,7 @@
               <showPercent val="0"/>
               <showBubbleSize val="0"/>
             </dLbl>
-            <numFmt formatCode="#,##0.0,&quot;K&quot;"/>
+            <numFmt formatCode="#,##0"/>
             <txPr>
               <a:bodyPr/>
               <a:p>
@@ -1879,7 +2010,7 @@
           <dLbls>
             <dLbl>
               <idx val="4"/>
-              <numFmt formatCode="#,##0.0,&quot;K&quot;"/>
+              <numFmt formatCode="#,##0"/>
               <dLblPos val="t"/>
               <showLegendKey val="0"/>
               <showVal val="1"/>
@@ -1888,7 +2019,7 @@
               <showPercent val="0"/>
               <showBubbleSize val="0"/>
             </dLbl>
-            <numFmt formatCode="#,##0.0,&quot;K&quot;"/>
+            <numFmt formatCode="#,##0"/>
             <txPr>
               <a:bodyPr/>
               <a:p>
@@ -1925,8 +2056,131 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <tx>
+            <v>Total (label)</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <txPr>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0">
+                    <a:solidFill>
+                      <a:srgbClr val="0B0B0B"/>
+                    </a:solidFill>
+                    <a:latin typeface="Aptos Narrow"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="900" b="1" i="0">
+                  <a:solidFill>
+                    <a:srgbClr val="0B0B0B"/>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="t"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+          </dLbls>
+          <val>
+            <numRef>
+              <f>'Chart Data'!$B$14:$F$14</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
         <axId val="10"/>
         <axId val="200"/>
+      </lineChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <tx>
+            <v>Total (label)</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <txPr>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0">
+                    <a:solidFill>
+                      <a:srgbClr val="0B0B0B"/>
+                    </a:solidFill>
+                    <a:latin typeface="Aptos Narrow"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="900" b="1" i="0">
+                  <a:solidFill>
+                    <a:srgbClr val="0B0B0B"/>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="t"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+          </dLbls>
+          <val>
+            <numRef>
+              <f>'Chart Data'!$B$15:$F$15</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
       </lineChart>
       <catAx>
         <axId val="10"/>
@@ -2049,6 +2303,14 @@
       </legendEntry>
       <legendEntry>
         <idx val="1"/>
+        <delete val="1"/>
+      </legendEntry>
+      <legendEntry>
+        <idx val="7"/>
+        <delete val="1"/>
+      </legendEntry>
+      <legendEntry>
+        <idx val="8"/>
         <delete val="1"/>
       </legendEntry>
       <layout>
@@ -2454,8 +2716,131 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <tx>
+            <v>Total (label)</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <txPr>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0">
+                    <a:solidFill>
+                      <a:srgbClr val="0B0B0B"/>
+                    </a:solidFill>
+                    <a:latin typeface="Aptos Narrow"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="900" b="1" i="0">
+                  <a:solidFill>
+                    <a:srgbClr val="0B0B0B"/>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="t"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+          </dLbls>
+          <val>
+            <numRef>
+              <f>'Chart Data'!$B$14:$F$14</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
         <axId val="10"/>
         <axId val="200"/>
+      </lineChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <tx>
+            <v>Total (label)</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <txPr>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0">
+                    <a:solidFill>
+                      <a:srgbClr val="0B0B0B"/>
+                    </a:solidFill>
+                    <a:latin typeface="Aptos Narrow"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="900" b="1" i="0">
+                  <a:solidFill>
+                    <a:srgbClr val="0B0B0B"/>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="t"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+          </dLbls>
+          <val>
+            <numRef>
+              <f>'Chart Data'!$B$15:$F$15</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
       </lineChart>
       <catAx>
         <axId val="10"/>
@@ -2578,6 +2963,14 @@
       </legendEntry>
       <legendEntry>
         <idx val="1"/>
+        <delete val="1"/>
+      </legendEntry>
+      <legendEntry>
+        <idx val="7"/>
+        <delete val="1"/>
+      </legendEntry>
+      <legendEntry>
+        <idx val="8"/>
         <delete val="1"/>
       </legendEntry>
       <overlay val="0"/>
@@ -2954,6 +3347,65 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <v>Total (label)</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <txPr>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0">
+                    <a:solidFill>
+                      <a:srgbClr val="0B0B0B"/>
+                    </a:solidFill>
+                    <a:latin typeface="Aptos Narrow"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="900" b="1" i="0">
+                  <a:solidFill>
+                    <a:srgbClr val="0B0B0B"/>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="t"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+          </dLbls>
+          <val>
+            <numRef>
+              <f>'Chart Data'!$B$14:$F$14</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -3058,6 +3510,10 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <legendEntry>
+        <idx val="5"/>
+        <delete val="1"/>
+      </legendEntry>
       <overlay val="0"/>
       <txPr>
         <a:bodyPr/>

</xml_diff>

<commit_message>
Draw demand line continuously through the last quarter, no endpoint dot
The per-point endpoint marker override also broke the final line segment
in Excel; removing it lets the line render straight through Q4'27. Same
fix applied to the capacity reference line on the funnel sheet. Labels
and everything else unchanged.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014fnah7533XZizagq8i6MTs
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/Supplier_Capacity_Inputs.xlsx
+++ b/PVA second supplier initiative/Supplier_Capacity_Inputs.xlsx
@@ -932,13 +932,13 @@
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008300"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF459428"/>
+      <rgbColor rgb="FF7F7F7F"/>
       <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF7F7F7F"/>
+      <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBFBF"/>
       <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF889AAA"/>
-      <rgbColor rgb="FFA02B93"/>
+      <rgbColor rgb="FF8B8B8B"/>
+      <rgbColor rgb="FFE34948"/>
       <rgbColor rgb="FFF7F7F7"/>
       <rgbColor rgb="FFE7E7E7"/>
       <rgbColor rgb="FF660066"/>
@@ -959,7 +959,7 @@
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FFB3B3B3"/>
       <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FF8B8B8B"/>
+      <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF2A78D6"/>
       <rgbColor rgb="FF33CCCC"/>
@@ -974,7 +974,7 @@
       <rgbColor rgb="FF0B0B0B"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FFE34948"/>
+      <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF4A3AA7"/>
       <rgbColor rgb="FF404040"/>
     </indexedColors>
@@ -1305,29 +1305,6 @@
               </a:ln>
             </spPr>
           </marker>
-          <dPt>
-            <idx val="4"/>
-            <marker>
-              <symbol val="circle"/>
-              <size val="7"/>
-              <spPr>
-                <a:solidFill>
-                  <a:srgbClr val="0B0B0B"/>
-                </a:solidFill>
-                <a:ln w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                  <a:prstDash val="solid"/>
-                </a:ln>
-              </spPr>
-            </marker>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
           <dLbls>
             <dLbl>
               <idx val="4"/>
@@ -1984,29 +1961,6 @@
               </a:ln>
             </spPr>
           </marker>
-          <dPt>
-            <idx val="4"/>
-            <marker>
-              <symbol val="circle"/>
-              <size val="7"/>
-              <spPr>
-                <a:solidFill>
-                  <a:srgbClr val="0B0B0B"/>
-                </a:solidFill>
-                <a:ln w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                  <a:prstDash val="solid"/>
-                </a:ln>
-              </spPr>
-            </marker>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
           <dLbls>
             <dLbl>
               <idx val="4"/>
@@ -2686,29 +2640,6 @@
               </a:ln>
             </spPr>
           </marker>
-          <dPt>
-            <idx val="4"/>
-            <marker>
-              <symbol val="circle"/>
-              <size val="7"/>
-              <spPr>
-                <a:solidFill>
-                  <a:srgbClr val="0B0B0B"/>
-                </a:solidFill>
-                <a:ln w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                  <a:prstDash val="solid"/>
-                </a:ln>
-              </spPr>
-            </marker>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
           <val>
             <numRef>
               <f>'Chart Data'!$B$21:$F$21</f>
@@ -3275,29 +3206,6 @@
               </a:ln>
             </spPr>
           </marker>
-          <dPt>
-            <idx val="4"/>
-            <marker>
-              <symbol val="circle"/>
-              <size val="7"/>
-              <spPr>
-                <a:solidFill>
-                  <a:srgbClr val="0B0B0B"/>
-                </a:solidFill>
-                <a:ln w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                  <a:prstDash val="solid"/>
-                </a:ln>
-              </spPr>
-            </marker>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
           <dLbls>
             <dLbl>
               <idx val="4"/>
@@ -4205,29 +4113,6 @@
               </a:ln>
             </spPr>
           </marker>
-          <dPt>
-            <idx val="4"/>
-            <marker>
-              <symbol val="circle"/>
-              <size val="6"/>
-              <spPr>
-                <a:solidFill>
-                  <a:srgbClr val="999999"/>
-                </a:solidFill>
-                <a:ln w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                  <a:prstDash val="solid"/>
-                </a:ln>
-              </spPr>
-            </marker>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
           <dLbls>
             <dLbl>
               <idx val="4"/>

</xml_diff>